<commit_message>
fix: repair skill stone picker and correct Dimension matchups
</commit_message>
<xml_diff>
--- a/docs/Seer_Type_Chart.xlsx
+++ b/docs/Seer_Type_Chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\seervote\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\seervote\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F575E8-2E5F-42E4-88E3-EA22EF21FD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516F30FA-B8A7-425A-BB10-80913A5A0261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -255,10 +255,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>冰、王、混沌、邪靈、輪迴</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>草、飛行、神秘、龍、虛空</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -344,6 +340,10 @@
   </si>
   <si>
     <t>戰鬥、神秘、自然</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>冰、王、神靈、混沌、輪迴</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -822,7 +822,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>31</v>
@@ -948,7 +948,7 @@
         <v>14</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>49</v>
@@ -1049,7 +1049,7 @@
         <v>65</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>64</v>
@@ -1060,10 +1060,10 @@
         <v>22</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>68</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>32</v>
@@ -1074,13 +1074,13 @@
         <v>23</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1088,10 +1088,10 @@
         <v>24</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>32</v>
@@ -1102,10 +1102,10 @@
         <v>25</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>75</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>32</v>
@@ -1116,13 +1116,13 @@
         <v>26</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="D24" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
@@ -1130,10 +1130,10 @@
         <v>27</v>
       </c>
       <c r="B25" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>85</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>32</v>
@@ -1144,10 +1144,10 @@
         <v>28</v>
       </c>
       <c r="B26" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>80</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>32</v>
@@ -1158,10 +1158,10 @@
         <v>29</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>82</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>32</v>
@@ -1172,10 +1172,10 @@
         <v>30</v>
       </c>
       <c r="B28" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>32</v>

</xml_diff>